<commit_message>
Refactor partner registration flow and clean up internal Zone labels
</commit_message>
<xml_diff>
--- a/backend/data/specialists_export.xlsx
+++ b/backend/data/specialists_export.xlsx
@@ -479,11 +479,7 @@
           <t>Я працюю в цій сфері більше 15 років і маю більше 30 успішних кейсів</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>verified</t>
@@ -516,11 +512,7 @@
           <t>Аароллдддллорпропроо</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>verified</t>

</xml_diff>